<commit_message>
updated plots with updated ledger entries
</commit_message>
<xml_diff>
--- a/results/Data/gcr_resilience_vulnerability_evidence_ledger.xlsx
+++ b/results/Data/gcr_resilience_vulnerability_evidence_ledger.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Ledger" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ledger!$A$1:$J$159</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ledger!$A$1:$J$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ledger!$A$1:$J$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ledger!$A$1:$J$158</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
   <extLst>
@@ -452,343 +452,343 @@
     <t xml:space="preserve">Manheim &amp; Denkenberger 2020</t>
   </si>
   <si>
+    <t>Sweden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strong health systems; high GHS Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denmark/Finland/Norway/Sweden in highest GHS group</t>
+  </si>
+  <si>
+    <t>Finland</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very reliant on trade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Under nuclear umbrella - elevated targeting risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High GHS Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aged population</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Korea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HEMP protection efforts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pry 2017</t>
+  </si>
+  <si>
+    <t>§3.3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very trade-dependent</t>
+  </si>
+  <si>
+    <t>Taiwan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">United Kingdom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Democratic </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pry 2012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In high-likelihood space-weather damage zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some HEMP protection</t>
+  </si>
+  <si>
+    <t>mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pry 2017; House of Commons Defence Committee 2012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuclear weapon state / NATO - elevated direct-targeting risk</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Well-organised non-island jurisdiction limiting pandemic harms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High-latitude cooling</t>
+  </si>
+  <si>
+    <t>Cuba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resilience under limited trade/reduced agricultural inputs</t>
+  </si>
+  <si>
+    <t>Vanuatu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ample food production</t>
+  </si>
+  <si>
+    <t xml:space="preserve">§3.1.3, §3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High above sea level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could maintain traditional life</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lacks infrastructure/manufacturing to sustain industrial society without trade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solomon Islands</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large food excess</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lacks infrastructure/manufacturing without trade</t>
+  </si>
+  <si>
+    <t>Indonesia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk from social/political instability during ASRS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learned volcano resilience</t>
+  </si>
+  <si>
+    <t>Peru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resilient location for climate/food impacts (equatorial upwelling, seaweed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jehn et al. 2024; Scherrer et al. 2020</t>
+  </si>
+  <si>
+    <t>Bolivia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equatorial Andes - prime food stockpile siting (La Paz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maher &amp; Baum 2013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stockpile location, not population resilience per se</t>
+  </si>
+  <si>
+    <t>Colombia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equatorial Andes - prime food stockpile siting (Pasto)</t>
+  </si>
+  <si>
+    <t>Philippines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">United States</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuclear weapon state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coupe et al. 2019; Denkenberger et al. 2017; Jehn et al. 2024; Mills et al. 2014; Scherrer et al. 2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forecasting capability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fry 2012; Johnson et al. 2016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grid hardening</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High GHS Index but poor outcomes (political will, cohesion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lyu et al. 2023; Nuzzo &amp; Ledesma 2023</t>
+  </si>
+  <si>
+    <t>§3.4.3</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochman et al. 2022; Jehn et al. 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Food/trade exposure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grid hardening against geomagnetic storms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Johnson et al. 2016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cameron et al. 2019; author synthesis</t>
+  </si>
+  <si>
+    <t>Russia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coupe et al. 2019; Early &amp; Asal 2014; Hochman et al. 2022</t>
+  </si>
+  <si>
+    <t>Ukraine</t>
+  </si>
+  <si>
+    <t>cyber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reverted grid to manual control after cyberattack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Knake 2017</t>
+  </si>
+  <si>
+    <t>§3.3.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At risk from Russia - elevated direct-targeting risk</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fared reasonably well as climate refuge after Toba supereruption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black et al. 2021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deep-time analogue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuclear weapon state - elevated direct-targeting risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">North Korea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named in nuclear-winter at-risk list; nuclear weapon state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochman et al. 2022</t>
+  </si>
+  <si>
+    <t>Israel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named in nuclear-winter at-risk list; nuclear weapon state / conflict</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Early &amp; Asal 2014</t>
+  </si>
+  <si>
+    <t>Iran</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named in at-risk list; conflict with Israel/US - targeting risk</t>
+  </si>
+  <si>
+    <t>Pakistan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named in at-risk list; nuclear weapon state</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central Europe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High cooling / agricultural exposure in nuclear winter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jehn et al. 2024, 2025a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eastern Europe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coupe et al. 2019; Jehn et al. 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southern Africa &amp; South America</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparatively resilient to climate/food impacts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mills et al. 2014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mediterranean climate zones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Climate-zone vulnerability in nuclear winter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grime 1986</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asian monsoon regions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monsoon disruption vulnerability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sub-Saharan Africa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deep-time analogue; paired with India in text</t>
+  </si>
+  <si>
+    <t>Tuvalu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small island: sea-level rise, tsunami &amp; NEO exposure; not self-sufficient</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boyd et al. 2023; Wilson et al. 2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marshall Islands</t>
+  </si>
+  <si>
+    <t>Ireland</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northern Germany in high-likelihood space-weather damage zone</t>
+  </si>
+  <si>
+    <t>Baltics</t>
+  </si>
+  <si>
     <t>Scandinavia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strong health systems; high GHS Index</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Denmark/Finland/Norway/Sweden in highest GHS group</t>
-  </si>
-  <si>
-    <t>Japan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Very reliant on trade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Under nuclear umbrella - elevated targeting risk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High GHS Index</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aged population</t>
-  </si>
-  <si>
-    <t xml:space="preserve">South Korea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEMP protection efforts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pry 2017</t>
-  </si>
-  <si>
-    <t>§3.3.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Very trade-dependent</t>
-  </si>
-  <si>
-    <t>Taiwan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Large industrial base</t>
-  </si>
-  <si>
-    <t xml:space="preserve">United Kingdom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Democratic </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pry 2012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In high-likelihood space-weather damage zone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Some HEMP protection</t>
-  </si>
-  <si>
-    <t>mixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pry 2017; House of Commons Defence Committee 2012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nuclear weapon state / NATO - elevated direct-targeting risk</t>
-  </si>
-  <si>
-    <t>China</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Well-organised non-island jurisdiction limiting pandemic harms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High-latitude cooling</t>
-  </si>
-  <si>
-    <t>Cuba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resilience under limited trade/reduced agricultural inputs</t>
-  </si>
-  <si>
-    <t>Vanuatu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ample food production</t>
-  </si>
-  <si>
-    <t xml:space="preserve">§3.1.3, §3.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High above sea level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Could maintain traditional life</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lacks infrastructure/manufacturing to sustain industrial society without trade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solomon Islands</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Large food excess</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lacks infrastructure/manufacturing without trade</t>
-  </si>
-  <si>
-    <t>Indonesia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Risk from social/political instability during ASRS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Learned volcano resilience</t>
-  </si>
-  <si>
-    <t>Peru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resilient location for climate/food impacts (equatorial upwelling, seaweed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jehn et al. 2024; Scherrer et al. 2020</t>
-  </si>
-  <si>
-    <t>Bolivia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equatorial Andes - prime food stockpile siting (La Paz)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maher &amp; Baum 2013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stockpile location, not population resilience per se</t>
-  </si>
-  <si>
-    <t>Colombia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equatorial Andes - prime food stockpile siting (Pasto)</t>
-  </si>
-  <si>
-    <t>Philippines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">United States</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nuclear weapon state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coupe et al. 2019; Denkenberger et al. 2017; Jehn et al. 2024; Mills et al. 2014; Scherrer et al. 2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forecasting capability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fry 2012; Johnson et al. 2016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grid hardening</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High GHS Index but poor outcomes (political will, cohesion)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lyu et al. 2023; Nuzzo &amp; Ledesma 2023</t>
-  </si>
-  <si>
-    <t>§3.4.3</t>
-  </si>
-  <si>
-    <t>Canada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hochman et al. 2022; Jehn et al. 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Food/trade exposure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grid hardening against geomagnetic storms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Johnson et al. 2016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cameron et al. 2019; author synthesis</t>
-  </si>
-  <si>
-    <t>Russia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coupe et al. 2019; Early &amp; Asal 2014; Hochman et al. 2022</t>
-  </si>
-  <si>
-    <t>Ukraine</t>
-  </si>
-  <si>
-    <t>cyber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reverted grid to manual control after cyberattack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Knake 2017</t>
-  </si>
-  <si>
-    <t>§3.3.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">At risk from Russia - elevated direct-targeting risk</t>
-  </si>
-  <si>
-    <t>India</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fared reasonably well as climate refuge after Toba supereruption</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Black et al. 2021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deep-time analogue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nuclear weapon state - elevated direct-targeting risk</t>
-  </si>
-  <si>
-    <t>Sweden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">North Korea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Named in nuclear-winter at-risk list; nuclear weapon state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hochman et al. 2022</t>
-  </si>
-  <si>
-    <t>Israel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Named in nuclear-winter at-risk list; nuclear weapon state / conflict</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Early &amp; Asal 2014</t>
-  </si>
-  <si>
-    <t>Iran</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Named in at-risk list; conflict with Israel/US - targeting risk</t>
-  </si>
-  <si>
-    <t>Pakistan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Named in at-risk list; nuclear weapon state</t>
-  </si>
-  <si>
-    <t>France</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Central Europe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High cooling / agricultural exposure in nuclear winter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jehn et al. 2024, 2025a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eastern Europe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coupe et al. 2019; Jehn et al. 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southern Africa &amp; South America</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comparatively resilient to climate/food impacts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mills et al. 2014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mediterranean climate zones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Climate-zone vulnerability in nuclear winter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grime 1986</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asian monsoon regions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monsoon disruption vulnerability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sub-Saharan Africa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deep-time analogue; paired with India in text</t>
-  </si>
-  <si>
-    <t>Tuvalu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small island: sea-level rise, tsunami &amp; NEO exposure; not self-sufficient</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boyd et al. 2023; Wilson et al. 2025)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marshall Islands</t>
-  </si>
-  <si>
-    <t>Ireland</t>
-  </si>
-  <si>
-    <t>Germany</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Northern Germany in high-likelihood space-weather damage zone</t>
-  </si>
-  <si>
-    <t>Baltics</t>
   </si>
   <si>
     <t xml:space="preserve">European Union</t>
@@ -872,16 +872,16 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.000000"/>
+      <sz val="11.000000"/>
       <name val="Arial"/>
     </font>
     <font>
       <sz val="11.000000"/>
+      <color rgb="FF9A1B1B"/>
       <name val="Arial"/>
     </font>
     <font>
       <sz val="10.000000"/>
-      <color rgb="FF9A1B1B"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1768,7 +1768,7 @@
         <v>14</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I9" s="2" t="s">
@@ -1804,7 +1804,7 @@
         <v>14</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I10" s="2" t="s">
@@ -1853,7 +1853,7 @@
       <c r="D12" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F12" s="3" t="s">
@@ -1888,7 +1888,7 @@
         <v>14</v>
       </c>
       <c r="G13" s="2"/>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="2" t="s">
         <v>48</v>
       </c>
       <c r="I13" s="2" t="s">
@@ -2055,7 +2055,7 @@
       <c r="D19" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F19" s="3" t="s">
@@ -2159,7 +2159,7 @@
       <c r="D23" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -2275,7 +2275,7 @@
       <c r="D27" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F27" s="3" t="s">
@@ -2303,7 +2303,7 @@
       <c r="D28" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E28" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F28" s="3" t="s">
@@ -2338,7 +2338,7 @@
         <v>14</v>
       </c>
       <c r="G29" s="2"/>
-      <c r="H29" s="6" t="s">
+      <c r="H29" s="2" t="s">
         <v>83</v>
       </c>
       <c r="I29" s="2" t="s">
@@ -2359,7 +2359,7 @@
       <c r="D30" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F30" s="4" t="s">
@@ -2445,7 +2445,7 @@
       <c r="D33" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E33" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F33" s="3" t="s">
@@ -2473,7 +2473,7 @@
       <c r="D34" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F34" s="3" t="s">
@@ -2501,7 +2501,7 @@
       <c r="D35" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="E35" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F35" s="4" t="s">
@@ -2616,7 +2616,7 @@
         <v>14</v>
       </c>
       <c r="G39" s="2"/>
-      <c r="H39" s="6" t="s">
+      <c r="H39" s="2" t="s">
         <v>83</v>
       </c>
       <c r="I39" s="2" t="s">
@@ -2670,7 +2670,7 @@
         <v>14</v>
       </c>
       <c r="G41" s="2"/>
-      <c r="H41" s="6" t="s">
+      <c r="H41" s="2" t="s">
         <v>104</v>
       </c>
       <c r="I41" s="2" t="s">
@@ -2696,7 +2696,7 @@
         <v>14</v>
       </c>
       <c r="G42" s="2"/>
-      <c r="H42" s="6" t="s">
+      <c r="H42" s="2" t="s">
         <v>106</v>
       </c>
       <c r="I42" s="2" t="s">
@@ -2722,7 +2722,7 @@
         <v>14</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="H43" s="6" t="s">
+      <c r="H43" s="2" t="s">
         <v>108</v>
       </c>
       <c r="I43" s="2" t="s">
@@ -2771,7 +2771,7 @@
       <c r="D45" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E45" s="7" t="s">
+      <c r="E45" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F45" s="3" t="s">
@@ -2799,7 +2799,7 @@
       <c r="D46" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E46" s="7" t="s">
+      <c r="E46" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F46" s="3" t="s">
@@ -2883,7 +2883,7 @@
       <c r="D49" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E49" s="7" t="s">
+      <c r="E49" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F49" s="3" t="s">
@@ -2911,7 +2911,7 @@
       <c r="D50" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E50" s="7" t="s">
+      <c r="E50" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F50" s="3" t="s">
@@ -2931,11 +2931,9 @@
         <v>115</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C51" s="2"/>
       <c r="D51" s="2" t="s">
         <v>116</v>
       </c>
@@ -3015,15 +3013,13 @@
         <v>115</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C54" s="2"/>
       <c r="D54" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E54" s="7" t="s">
+      <c r="E54" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F54" s="3" t="s">
@@ -3058,7 +3054,7 @@
         <v>14</v>
       </c>
       <c r="G55" s="2"/>
-      <c r="H55" s="6" t="s">
+      <c r="H55" s="2" t="s">
         <v>120</v>
       </c>
       <c r="I55" s="2" t="s">
@@ -3167,14 +3163,14 @@
       <c r="D59" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="E59" s="7" t="s">
+      <c r="E59" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G59" s="2"/>
-      <c r="H59" s="6" t="s">
+      <c r="H59" s="2" t="s">
         <v>48</v>
       </c>
       <c r="I59" s="2" t="s">
@@ -3195,7 +3191,7 @@
       <c r="D60" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E60" s="7" t="s">
+      <c r="E60" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F60" s="3" t="s">
@@ -3223,7 +3219,7 @@
       <c r="D61" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="E61" s="7" t="s">
+      <c r="E61" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F61" s="3" t="s">
@@ -3314,7 +3310,7 @@
         <v>14</v>
       </c>
       <c r="G64" s="2"/>
-      <c r="H64" s="6" t="s">
+      <c r="H64" s="2" t="s">
         <v>120</v>
       </c>
       <c r="I64" s="2" t="s">
@@ -3348,7 +3344,7 @@
       <c r="I65" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="J65" s="6" t="s">
+      <c r="J65" s="2" t="s">
         <v>135</v>
       </c>
     </row>
@@ -3372,7 +3368,7 @@
         <v>14</v>
       </c>
       <c r="G66" s="2"/>
-      <c r="H66" s="6" t="s">
+      <c r="H66" s="2" t="s">
         <v>137</v>
       </c>
       <c r="I66" s="2" t="s">
@@ -3441,13 +3437,11 @@
         <v>140</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C69" s="2"/>
       <c r="D69" s="2" t="s">
-        <v>141</v>
+        <v>20</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>13</v>
@@ -3457,79 +3451,79 @@
       </c>
       <c r="G69" s="2"/>
       <c r="H69" s="2" t="s">
-        <v>142</v>
+        <v>21</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="J69" s="2"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C70" s="2"/>
       <c r="D70" s="2" t="s">
-        <v>144</v>
+        <v>22</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F70" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G70" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="H70" s="2"/>
+      <c r="F70" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G70" s="2"/>
+      <c r="H70" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="I70" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="J70" s="2" t="s">
-        <v>145</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="J70" s="2"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C71" s="2"/>
+        <v>58</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="D71" s="2" t="s">
-        <v>12</v>
+        <v>89</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F71" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G71" s="2"/>
-      <c r="H71" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="F71" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H71" s="2"/>
       <c r="I71" s="2" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="J71" s="2"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C72" s="2"/>
+        <v>58</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="D72" s="2" t="s">
-        <v>18</v>
+        <v>141</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>13</v>
@@ -3539,85 +3533,93 @@
       </c>
       <c r="G72" s="2"/>
       <c r="H72" s="2" t="s">
-        <v>19</v>
+        <v>142</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="J72" s="2"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C73" s="2"/>
+        <v>58</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="D73" s="2" t="s">
-        <v>20</v>
+        <v>144</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F73" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G73" s="2"/>
-      <c r="H73" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="F73" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H73" s="2"/>
       <c r="I73" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J73" s="2"/>
+        <v>62</v>
+      </c>
+      <c r="J73" s="2" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="s">
         <v>146</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C74" s="2"/>
+        <v>58</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="D74" s="2" t="s">
-        <v>22</v>
+        <v>144</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F74" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G74" s="2"/>
-      <c r="H74" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="F74" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H74" s="2"/>
       <c r="I74" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J74" s="2"/>
+        <v>62</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E75" s="7" t="s">
-        <v>43</v>
+        <v>12</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F75" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G75" s="2"/>
       <c r="H75" s="2" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="I75" s="2" t="s">
         <v>16</v>
@@ -3626,44 +3628,40 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>38</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C76" s="2"/>
       <c r="D76" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="E76" s="7" t="s">
-        <v>43</v>
+        <v>18</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F76" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G76" s="2"/>
       <c r="H76" s="2" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="I76" s="2" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="J76" s="2"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>46</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C77" s="2"/>
       <c r="D77" s="2" t="s">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>13</v>
@@ -3672,26 +3670,24 @@
         <v>14</v>
       </c>
       <c r="G77" s="2"/>
-      <c r="H77" s="6" t="s">
-        <v>83</v>
+      <c r="H77" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="I77" s="2" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="J77" s="2"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C78" s="2"/>
       <c r="D78" s="2" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>13</v>
@@ -3700,56 +3696,54 @@
         <v>14</v>
       </c>
       <c r="G78" s="2"/>
-      <c r="H78" s="6" t="s">
-        <v>55</v>
+      <c r="H78" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="I78" s="2" t="s">
-        <v>87</v>
+        <v>16</v>
       </c>
       <c r="J78" s="2"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>59</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C79" s="2"/>
       <c r="D79" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F79" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G79" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="H79" s="2"/>
+        <v>148</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G79" s="2"/>
+      <c r="H79" s="2" t="s">
+        <v>129</v>
+      </c>
       <c r="I79" s="2" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="J79" s="2"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="E80" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E80" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F80" s="3" t="s">
@@ -3760,69 +3754,69 @@
         <v>44</v>
       </c>
       <c r="I80" s="2" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="J80" s="2"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>133</v>
+        <v>46</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>152</v>
+        <v>82</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F81" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G81" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="H81" s="2"/>
+      <c r="F81" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G81" s="2"/>
+      <c r="H81" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="I81" s="2" t="s">
-        <v>154</v>
+        <v>84</v>
       </c>
       <c r="J81" s="2"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>149</v>
+        <v>54</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F82" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G82" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="H82" s="2"/>
+      <c r="F82" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G82" s="2"/>
+      <c r="H82" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="I82" s="2" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="J82" s="2"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>58</v>
@@ -3831,18 +3825,18 @@
         <v>59</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E83" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F83" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G83" s="2"/>
-      <c r="H83" s="2" t="s">
-        <v>129</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H83" s="2"/>
       <c r="I83" s="2" t="s">
         <v>62</v>
       </c>
@@ -3850,7 +3844,7 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>58</v>
@@ -3859,9 +3853,9 @@
         <v>59</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="E84" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="E84" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F84" s="3" t="s">
@@ -3878,159 +3872,167 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C85" s="2"/>
+        <v>52</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>133</v>
+      </c>
       <c r="D85" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F85" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G85" s="2"/>
-      <c r="H85" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="F85" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H85" s="2"/>
       <c r="I85" s="2" t="s">
-        <v>16</v>
+        <v>155</v>
       </c>
       <c r="J85" s="2"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C86" s="2"/>
+        <v>58</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="D86" s="2" t="s">
-        <v>18</v>
+        <v>150</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F86" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G86" s="2"/>
-      <c r="H86" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="F86" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H86" s="2"/>
       <c r="I86" s="2" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="J86" s="2"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D87" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B87" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>13</v>
+      <c r="E87" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F87" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G87" s="2"/>
       <c r="H87" s="2" t="s">
-        <v>21</v>
+        <v>129</v>
       </c>
       <c r="I87" s="2" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="J87" s="2"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C88" s="2"/>
+        <v>58</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="D88" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>13</v>
+        <v>151</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G88" s="2"/>
       <c r="H88" s="2" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="I88" s="2" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="J88" s="2"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C89" s="2"/>
+        <v>52</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>133</v>
+      </c>
       <c r="D89" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H89" s="2"/>
+      <c r="I89" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="E89" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F89" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G89" s="2"/>
-      <c r="H89" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="I89" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="J89" s="2"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>133</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C90" s="2"/>
       <c r="D90" s="2" t="s">
-        <v>152</v>
+        <v>18</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F90" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G90" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="H90" s="2"/>
+      <c r="F90" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G90" s="2"/>
+      <c r="H90" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="I90" s="2" t="s">
-        <v>154</v>
+        <v>16</v>
       </c>
       <c r="J90" s="2"/>
     </row>
@@ -4043,7 +4045,7 @@
       </c>
       <c r="C91" s="2"/>
       <c r="D91" s="2" t="s">
-        <v>18</v>
+        <v>159</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>13</v>
@@ -4053,7 +4055,7 @@
       </c>
       <c r="G91" s="2"/>
       <c r="H91" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I91" s="2" t="s">
         <v>16</v>
@@ -4065,24 +4067,26 @@
         <v>158</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C92" s="2"/>
+        <v>52</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="D92" s="2" t="s">
-        <v>159</v>
+        <v>54</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F92" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G92" s="2"/>
-      <c r="H92" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="F92" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="H92" s="2"/>
       <c r="I92" s="2" t="s">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="J92" s="2"/>
     </row>
@@ -4097,16 +4101,16 @@
         <v>53</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E93" s="2" t="s">
-        <v>13</v>
+        <v>161</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F93" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>160</v>
+        <v>86</v>
       </c>
       <c r="H93" s="2"/>
       <c r="I93" s="2" t="s">
@@ -4122,23 +4126,23 @@
         <v>52</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>53</v>
+        <v>133</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="E94" s="7" t="s">
-        <v>43</v>
+        <v>162</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="H94" s="2"/>
       <c r="I94" s="2" t="s">
-        <v>56</v>
+        <v>155</v>
       </c>
       <c r="J94" s="2"/>
     </row>
@@ -4147,54 +4151,54 @@
         <v>158</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>133</v>
+        <v>38</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="E95" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G95" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="H95" s="2"/>
+        <v>165</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F95" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G95" s="2"/>
+      <c r="H95" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="I95" s="2" t="s">
-        <v>154</v>
+        <v>41</v>
       </c>
       <c r="J95" s="2"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E96" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F96" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G96" s="2"/>
-      <c r="H96" s="2" t="s">
-        <v>44</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H96" s="2"/>
       <c r="I96" s="2" t="s">
-        <v>41</v>
+        <v>87</v>
       </c>
       <c r="J96" s="2"/>
     </row>
@@ -4206,10 +4210,10 @@
         <v>52</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>53</v>
+        <v>133</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>54</v>
+        <v>153</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>13</v>
@@ -4218,11 +4222,11 @@
         <v>26</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H97" s="2"/>
       <c r="I97" s="2" t="s">
-        <v>87</v>
+        <v>155</v>
       </c>
       <c r="J97" s="2"/>
     </row>
@@ -4231,13 +4235,13 @@
         <v>166</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>133</v>
+        <v>59</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>13</v>
@@ -4246,11 +4250,11 @@
         <v>26</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>153</v>
+        <v>69</v>
       </c>
       <c r="H98" s="2"/>
       <c r="I98" s="2" t="s">
-        <v>154</v>
+        <v>70</v>
       </c>
       <c r="J98" s="2"/>
     </row>
@@ -4259,82 +4263,82 @@
         <v>166</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="E99" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F99" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G99" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="H99" s="2"/>
+        <v>168</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F99" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G99" s="2"/>
+      <c r="H99" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="I99" s="2" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="J99" s="2"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="E100" s="7" t="s">
-        <v>43</v>
+        <v>170</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G100" s="2"/>
       <c r="H100" s="2" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="I100" s="2" t="s">
-        <v>41</v>
+        <v>93</v>
       </c>
       <c r="J100" s="2"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C101" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F101" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G101" s="2"/>
-      <c r="H101" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="F101" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H101" s="2"/>
       <c r="I101" s="2" t="s">
-        <v>93</v>
+        <v>173</v>
       </c>
       <c r="J101" s="2"/>
     </row>
@@ -4349,18 +4353,18 @@
         <v>24</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E102" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F102" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G102" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="H102" s="2"/>
+      <c r="F102" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G102" s="2"/>
+      <c r="H102" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="I102" s="2" t="s">
         <v>173</v>
       </c>
@@ -4377,18 +4381,18 @@
         <v>24</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F103" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G103" s="2"/>
-      <c r="H103" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="F103" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G103" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H103" s="2"/>
       <c r="I103" s="2" t="s">
         <v>173</v>
       </c>
@@ -4405,10 +4409,10 @@
         <v>24</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="E104" s="2" t="s">
-        <v>13</v>
+        <v>176</v>
+      </c>
+      <c r="E104" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F104" s="4" t="s">
         <v>26</v>
@@ -4418,13 +4422,13 @@
       </c>
       <c r="H104" s="2"/>
       <c r="I104" s="2" t="s">
-        <v>173</v>
+        <v>28</v>
       </c>
       <c r="J104" s="2"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>23</v>
@@ -4433,20 +4437,20 @@
         <v>24</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E105" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F105" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G105" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="H105" s="2"/>
+        <v>174</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G105" s="2"/>
+      <c r="H105" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="I105" s="2" t="s">
-        <v>28</v>
+        <v>173</v>
       </c>
       <c r="J105" s="2"/>
     </row>
@@ -4461,18 +4465,18 @@
         <v>24</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F106" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G106" s="2"/>
-      <c r="H106" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="F106" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G106" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H106" s="2"/>
       <c r="I106" s="2" t="s">
         <v>173</v>
       </c>
@@ -4489,10 +4493,10 @@
         <v>24</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="E107" s="2" t="s">
-        <v>13</v>
+        <v>179</v>
+      </c>
+      <c r="E107" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F107" s="4" t="s">
         <v>26</v>
@@ -4502,13 +4506,13 @@
       </c>
       <c r="H107" s="2"/>
       <c r="I107" s="2" t="s">
-        <v>173</v>
+        <v>28</v>
       </c>
       <c r="J107" s="2"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>23</v>
@@ -4517,18 +4521,18 @@
         <v>24</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="E108" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="E108" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F108" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G108" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="H108" s="2"/>
+      <c r="F108" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G108" s="2"/>
+      <c r="H108" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="I108" s="2" t="s">
         <v>28</v>
       </c>
@@ -4542,66 +4546,66 @@
         <v>23</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E109" s="7" t="s">
-        <v>43</v>
+        <v>182</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F109" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G109" s="2"/>
       <c r="H109" s="2" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="I109" s="2" t="s">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="J109" s="2"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F110" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G110" s="2"/>
-      <c r="H110" s="6" t="s">
-        <v>83</v>
-      </c>
+      <c r="F110" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G110" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H110" s="2"/>
       <c r="I110" s="2" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="J110" s="2"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>13</v>
@@ -4610,17 +4614,19 @@
         <v>26</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="H111" s="2"/>
       <c r="I111" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="J111" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="J111" s="2" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>23</v>
@@ -4629,7 +4635,7 @@
         <v>24</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>13</v>
@@ -4650,59 +4656,57 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F113" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G113" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="H113" s="2"/>
+      <c r="F113" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G113" s="2"/>
+      <c r="H113" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="I113" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J113" s="2" t="s">
-        <v>189</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="J113" s="2"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F114" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G114" s="2"/>
-      <c r="H114" s="6" t="s">
-        <v>83</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="E114" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H114" s="2"/>
       <c r="I114" s="2" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="J114" s="2"/>
     </row>
@@ -4717,9 +4721,9 @@
         <v>38</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="E115" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E115" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F115" s="4" t="s">
@@ -4742,23 +4746,23 @@
         <v>23</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="E116" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F116" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G116" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="H116" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G116" s="2"/>
+      <c r="H116" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="I116" s="2" t="s">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="J116" s="2"/>
     </row>
@@ -4767,26 +4771,26 @@
         <v>193</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>82</v>
+        <v>196</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F117" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G117" s="2"/>
-      <c r="H117" s="6" t="s">
-        <v>83</v>
-      </c>
+      <c r="F117" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G117" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="H117" s="2"/>
       <c r="I117" s="2" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="J117" s="2"/>
     </row>
@@ -4801,7 +4805,7 @@
         <v>53</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>13</v>
@@ -4829,16 +4833,16 @@
         <v>53</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>13</v>
+        <v>161</v>
+      </c>
+      <c r="E119" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F119" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>197</v>
+        <v>86</v>
       </c>
       <c r="H119" s="2"/>
       <c r="I119" s="2" t="s">
@@ -4854,23 +4858,23 @@
         <v>52</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>53</v>
+        <v>133</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="E120" s="7" t="s">
-        <v>43</v>
+        <v>153</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F120" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>86</v>
+        <v>154</v>
       </c>
       <c r="H120" s="2"/>
       <c r="I120" s="2" t="s">
-        <v>56</v>
+        <v>155</v>
       </c>
       <c r="J120" s="2"/>
     </row>
@@ -4879,54 +4883,54 @@
         <v>193</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>133</v>
+        <v>59</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="E121" s="2" t="s">
-        <v>13</v>
+        <v>199</v>
+      </c>
+      <c r="E121" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F121" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G121" s="2" t="s">
-        <v>153</v>
+        <v>200</v>
       </c>
       <c r="H121" s="2"/>
       <c r="I121" s="2" t="s">
-        <v>154</v>
+        <v>201</v>
       </c>
       <c r="J121" s="2"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="E122" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E122" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F122" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G122" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="H122" s="2"/>
       <c r="I122" s="2" t="s">
-        <v>201</v>
+        <v>41</v>
       </c>
       <c r="J122" s="2"/>
     </row>
@@ -4941,9 +4945,9 @@
         <v>38</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="E123" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="E123" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F123" s="4" t="s">
@@ -4963,26 +4967,26 @@
         <v>202</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="E124" s="7" t="s">
-        <v>43</v>
+        <v>205</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F124" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="H124" s="2"/>
       <c r="I124" s="2" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="J124" s="2"/>
     </row>
@@ -4997,16 +5001,16 @@
         <v>53</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="E125" s="2" t="s">
-        <v>13</v>
+        <v>161</v>
+      </c>
+      <c r="E125" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F125" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>206</v>
+        <v>86</v>
       </c>
       <c r="H125" s="2"/>
       <c r="I125" s="2" t="s">
@@ -5019,54 +5023,54 @@
         <v>202</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="E126" s="7" t="s">
-        <v>43</v>
+        <v>150</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F126" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>86</v>
+        <v>207</v>
       </c>
       <c r="H126" s="2"/>
       <c r="I126" s="2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="J126" s="2"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>13</v>
+        <v>194</v>
+      </c>
+      <c r="E127" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F127" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G127" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H127" s="2"/>
       <c r="I127" s="2" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="J127" s="2"/>
     </row>
@@ -5081,9 +5085,9 @@
         <v>38</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="E128" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E128" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F128" s="4" t="s">
@@ -5103,26 +5107,26 @@
         <v>208</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="E129" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="E129" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F129" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>209</v>
+        <v>86</v>
       </c>
       <c r="H129" s="2"/>
       <c r="I129" s="2" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="J129" s="2"/>
     </row>
@@ -5134,38 +5138,38 @@
         <v>52</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>53</v>
+        <v>133</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="E130" s="7" t="s">
-        <v>43</v>
+        <v>153</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F130" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>86</v>
+        <v>154</v>
       </c>
       <c r="H130" s="2"/>
       <c r="I130" s="2" t="s">
-        <v>56</v>
+        <v>155</v>
       </c>
       <c r="J130" s="2"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>133</v>
+        <v>211</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>152</v>
+        <v>212</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>13</v>
@@ -5174,11 +5178,11 @@
         <v>26</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>153</v>
+        <v>213</v>
       </c>
       <c r="H131" s="2"/>
       <c r="I131" s="2" t="s">
-        <v>154</v>
+        <v>214</v>
       </c>
       <c r="J131" s="2"/>
     </row>
@@ -5187,56 +5191,58 @@
         <v>210</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>211</v>
+        <v>38</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="E132" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F132" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G132" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="H132" s="2"/>
+        <v>215</v>
+      </c>
+      <c r="E132" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G132" s="2"/>
+      <c r="H132" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="I132" s="2" t="s">
-        <v>214</v>
+        <v>41</v>
       </c>
       <c r="J132" s="2"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="E133" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F133" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G133" s="2"/>
-      <c r="H133" s="2" t="s">
-        <v>44</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F133" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="H133" s="2"/>
       <c r="I133" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="J133" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="J133" s="2" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="s">
@@ -5246,53 +5252,51 @@
         <v>23</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="E134" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F134" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G134" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="H134" s="2"/>
+        <v>220</v>
+      </c>
+      <c r="E134" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G134" s="2"/>
+      <c r="H134" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="I134" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="J134" s="2" t="s">
-        <v>219</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="J134" s="2"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="s">
-        <v>216</v>
+        <v>143</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="E135" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F135" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G135" s="2"/>
-      <c r="H135" s="2" t="s">
-        <v>44</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F135" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="H135" s="2"/>
       <c r="I135" s="2" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="J135" s="2"/>
     </row>
@@ -5301,32 +5305,32 @@
         <v>221</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="E136" s="2" t="s">
-        <v>13</v>
+        <v>222</v>
+      </c>
+      <c r="E136" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F136" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>206</v>
+        <v>223</v>
       </c>
       <c r="H136" s="2"/>
       <c r="I136" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="J136" s="2"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>23</v>
@@ -5335,16 +5339,16 @@
         <v>38</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="E137" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="E137" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F137" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G137" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H137" s="2"/>
       <c r="I137" s="2" t="s">
@@ -5354,7 +5358,7 @@
     </row>
     <row r="138">
       <c r="A138" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>23</v>
@@ -5363,16 +5367,16 @@
         <v>38</v>
       </c>
       <c r="D138" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E138" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G138" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="E138" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F138" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G138" s="2" t="s">
-        <v>227</v>
       </c>
       <c r="H138" s="2"/>
       <c r="I138" s="2" t="s">
@@ -5382,7 +5386,7 @@
     </row>
     <row r="139">
       <c r="A139" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>23</v>
@@ -5391,16 +5395,16 @@
         <v>38</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E139" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="E139" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F139" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G139" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H139" s="2"/>
       <c r="I139" s="2" t="s">
@@ -5410,7 +5414,7 @@
     </row>
     <row r="140">
       <c r="A140" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>23</v>
@@ -5419,18 +5423,18 @@
         <v>38</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E140" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E140" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F140" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G140" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="H140" s="2"/>
+      <c r="F140" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G140" s="2"/>
+      <c r="H140" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="I140" s="2" t="s">
         <v>41</v>
       </c>
@@ -5447,18 +5451,18 @@
         <v>38</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E141" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E141" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F141" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G141" s="2"/>
-      <c r="H141" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="F141" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="H141" s="2"/>
       <c r="I141" s="2" t="s">
         <v>41</v>
       </c>
@@ -5466,7 +5470,7 @@
     </row>
     <row r="142">
       <c r="A142" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>23</v>
@@ -5475,16 +5479,16 @@
         <v>38</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="E142" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E142" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F142" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G142" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H142" s="2"/>
       <c r="I142" s="2" t="s">
@@ -5494,7 +5498,7 @@
     </row>
     <row r="143">
       <c r="A143" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>23</v>
@@ -5503,16 +5507,16 @@
         <v>38</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="E143" s="7" t="s">
-        <v>43</v>
+        <v>238</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F143" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G143" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="H143" s="2"/>
       <c r="I143" s="2" t="s">
@@ -5522,7 +5526,7 @@
     </row>
     <row r="144">
       <c r="A144" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B144" s="2" t="s">
         <v>23</v>
@@ -5531,16 +5535,16 @@
         <v>38</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="E144" s="2" t="s">
-        <v>13</v>
+        <v>241</v>
+      </c>
+      <c r="E144" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F144" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G144" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="H144" s="2"/>
       <c r="I144" s="2" t="s">
@@ -5550,7 +5554,7 @@
     </row>
     <row r="145">
       <c r="A145" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B145" s="2" t="s">
         <v>23</v>
@@ -5559,16 +5563,16 @@
         <v>38</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="E145" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="E145" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F145" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G145" s="2" t="s">
-        <v>243</v>
+        <v>108</v>
       </c>
       <c r="H145" s="2"/>
       <c r="I145" s="2" t="s">
@@ -5578,82 +5582,80 @@
     </row>
     <row r="146">
       <c r="A146" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="E146" s="7" t="s">
-        <v>43</v>
+        <v>217</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F146" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G146" s="2" t="s">
-        <v>108</v>
+        <v>218</v>
       </c>
       <c r="H146" s="2"/>
       <c r="I146" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="J146" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="J146" s="2" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C147" s="2" t="s">
-        <v>46</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C147" s="2"/>
       <c r="D147" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="E147" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F147" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G147" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="H147" s="2"/>
+        <v>248</v>
+      </c>
+      <c r="E147" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F147" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G147" s="2"/>
+      <c r="H147" s="2" t="s">
+        <v>249</v>
+      </c>
       <c r="I147" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="J147" s="2" t="s">
-        <v>247</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="J147" s="2"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C148" s="2"/>
       <c r="D148" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E148" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G148" s="2"/>
+      <c r="H148" s="2" t="s">
         <v>249</v>
-      </c>
-      <c r="E148" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F148" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G148" s="2"/>
-      <c r="H148" s="6" t="s">
-        <v>250</v>
       </c>
       <c r="I148" s="2" t="s">
         <v>95</v>
@@ -5662,33 +5664,35 @@
     </row>
     <row r="149">
       <c r="A149" s="2" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C149" s="2"/>
+        <v>52</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="D149" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E149" s="7" t="s">
-        <v>43</v>
+        <v>54</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F149" s="3" t="s">
         <v>14</v>
       </c>
       <c r="G149" s="2"/>
-      <c r="H149" s="6" t="s">
-        <v>250</v>
+      <c r="H149" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="I149" s="2" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="J149" s="2"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="s">
-        <v>232</v>
+        <v>251</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>52</v>
@@ -5697,18 +5701,18 @@
         <v>53</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E150" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F150" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G150" s="2"/>
-      <c r="H150" s="6" t="s">
-        <v>55</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="E150" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G150" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H150" s="2"/>
       <c r="I150" s="2" t="s">
         <v>87</v>
       </c>
@@ -5725,9 +5729,9 @@
         <v>53</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="E151" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="E151" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F151" s="4" t="s">
@@ -5744,7 +5748,7 @@
     </row>
     <row r="152">
       <c r="A152" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B152" s="2" t="s">
         <v>52</v>
@@ -5753,9 +5757,9 @@
         <v>53</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="E152" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="E152" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F152" s="4" t="s">
@@ -5783,7 +5787,7 @@
       <c r="D153" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E153" s="7" t="s">
+      <c r="E153" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F153" s="4" t="s">
@@ -5800,44 +5804,44 @@
     </row>
     <row r="154">
       <c r="A154" s="2" t="s">
-        <v>143</v>
+        <v>256</v>
       </c>
       <c r="B154" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="E154" s="7" t="s">
-        <v>43</v>
+        <v>257</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="F154" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G154" s="2" t="s">
-        <v>86</v>
+        <v>258</v>
       </c>
       <c r="H154" s="2"/>
       <c r="I154" s="2" t="s">
-        <v>87</v>
+        <v>259</v>
       </c>
       <c r="J154" s="2"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E155" s="2" t="s">
         <v>13</v>
@@ -5846,17 +5850,17 @@
         <v>26</v>
       </c>
       <c r="G155" s="2" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="H155" s="2"/>
       <c r="I155" s="2" t="s">
-        <v>259</v>
+        <v>70</v>
       </c>
       <c r="J155" s="2"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>58</v>
@@ -5865,26 +5869,26 @@
         <v>59</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="E156" s="2" t="s">
-        <v>13</v>
+        <v>264</v>
+      </c>
+      <c r="E156" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="F156" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G156" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="H156" s="2"/>
       <c r="I156" s="2" t="s">
-        <v>70</v>
+        <v>201</v>
       </c>
       <c r="J156" s="2"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>58</v>
@@ -5893,26 +5897,26 @@
         <v>59</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="E157" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="E157" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F157" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G157" s="2" t="s">
-        <v>265</v>
+        <v>65</v>
       </c>
       <c r="H157" s="2"/>
       <c r="I157" s="2" t="s">
-        <v>201</v>
+        <v>66</v>
       </c>
       <c r="J157" s="2"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>58</v>
@@ -5921,9 +5925,9 @@
         <v>59</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="E158" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="E158" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F158" s="4" t="s">
@@ -5938,100 +5942,72 @@
       </c>
       <c r="J158" s="2"/>
     </row>
-    <row r="159">
-      <c r="A159" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="B159" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C159" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D159" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="E159" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F159" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G159" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="H159" s="2"/>
-      <c r="I159" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="J159" s="2"/>
+    <row r="159" ht="14.25">
+      <c r="A159" s="7"/>
     </row>
     <row r="160" ht="14.25">
-      <c r="A160" s="2"/>
-    </row>
-    <row r="161" ht="14.25">
-      <c r="A161" s="2"/>
+      <c r="A160" s="7"/>
+    </row>
+    <row r="163" ht="14.25">
+      <c r="C163" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="D163" s="9"/>
     </row>
     <row r="164" ht="14.25">
-      <c r="C164" s="8" t="s">
-        <v>270</v>
-      </c>
+      <c r="C164" s="9"/>
       <c r="D164" s="9"/>
     </row>
     <row r="165" ht="14.25">
-      <c r="C165" s="9"/>
+      <c r="C165" s="10" t="s">
+        <v>271</v>
+      </c>
       <c r="D165" s="9"/>
     </row>
     <row r="166" ht="14.25">
-      <c r="C166" s="10" t="s">
-        <v>271</v>
-      </c>
-      <c r="D166" s="9"/>
+      <c r="C166" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D166" s="9" t="s">
+        <v>272</v>
+      </c>
     </row>
     <row r="167" ht="14.25">
       <c r="C167" s="9" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D167" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="168" ht="14.25">
-      <c r="C168" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D168" s="9" t="s">
-        <v>273</v>
-      </c>
+      <c r="C168" s="9"/>
+      <c r="D168" s="9"/>
     </row>
     <row r="169" ht="14.25">
       <c r="C169" s="9"/>
       <c r="D169" s="9"/>
     </row>
     <row r="170" ht="14.25">
-      <c r="C170" s="9"/>
+      <c r="C170" s="11" t="s">
+        <v>274</v>
+      </c>
       <c r="D170" s="9"/>
     </row>
     <row r="171" ht="14.25">
-      <c r="C171" s="11" t="s">
-        <v>274</v>
-      </c>
-      <c r="D171" s="9"/>
+      <c r="C171" s="9"/>
+      <c r="D171" s="9" t="s">
+        <v>275</v>
+      </c>
     </row>
     <row r="172" ht="14.25">
       <c r="C172" s="9"/>
       <c r="D172" s="9" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="173" ht="14.25">
-      <c r="C173" s="9"/>
-      <c r="D173" s="9" t="s">
         <v>276</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J159"/>
+  <autoFilter ref="A1:J158"/>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>

</xml_diff>